<commit_message>
- Change directories structure - Modify map visualization - and more
</commit_message>
<xml_diff>
--- a/data/100_fire_incidents.xlsx
+++ b/data/100_fire_incidents.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MetroSafe\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Me\UofL\Data Analytics &amp; System Optimization (DASO)\MetroSafe Drone-Project\MetroSafe-UofL_Drone_Optimization\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98565151-3B67-40E5-A740-2C62958191E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0635E0C3-4422-4B42-A628-B2AA3360E378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -402,7 +402,7 @@
     <t>latitude</t>
   </si>
   <si>
-    <t>longtitude</t>
+    <t>longitude</t>
   </si>
 </sst>
 </file>
@@ -721,16 +721,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E101"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>121</v>
       </c>
@@ -747,7 +747,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -764,7 +764,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -781,7 +781,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -798,7 +798,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -815,7 +815,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -832,7 +832,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -849,7 +849,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -866,7 +866,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -883,7 +883,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -900,7 +900,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -917,7 +917,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -934,7 +934,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -951,7 +951,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -968,7 +968,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -985,7 +985,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -1019,7 +1019,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -1036,7 +1036,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -1070,7 +1070,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -1087,7 +1087,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>30</v>
       </c>
@@ -1104,7 +1104,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -1138,7 +1138,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -1155,7 +1155,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>36</v>
       </c>
@@ -1172,7 +1172,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>38</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>40</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>26</v>
       </c>
@@ -1223,7 +1223,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>26</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>26</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>26</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>26</v>
       </c>
@@ -1291,7 +1291,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>26</v>
       </c>
@@ -1308,7 +1308,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>26</v>
       </c>
@@ -1325,7 +1325,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>26</v>
       </c>
@@ -1342,7 +1342,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>26</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1376,7 +1376,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>44</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>46</v>
       </c>
@@ -1410,7 +1410,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>48</v>
       </c>
@@ -1427,7 +1427,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>50</v>
       </c>
@@ -1444,7 +1444,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>52</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>52</v>
       </c>
@@ -1478,7 +1478,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>54</v>
       </c>
@@ -1495,7 +1495,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>56</v>
       </c>
@@ -1512,7 +1512,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>56</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>56</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>58</v>
       </c>
@@ -1563,7 +1563,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>60</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>62</v>
       </c>
@@ -1597,7 +1597,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>64</v>
       </c>
@@ -1614,7 +1614,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>66</v>
       </c>
@@ -1631,7 +1631,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>66</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>69</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>69</v>
       </c>
@@ -1682,7 +1682,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>71</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>71</v>
       </c>
@@ -1716,7 +1716,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>73</v>
       </c>
@@ -1733,7 +1733,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>73</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>73</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>73</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>73</v>
       </c>
@@ -1801,7 +1801,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>75</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>75</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>77</v>
       </c>
@@ -1852,7 +1852,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>79</v>
       </c>
@@ -1869,7 +1869,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>79</v>
       </c>
@@ -1886,7 +1886,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>79</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>81</v>
       </c>
@@ -1920,7 +1920,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>83</v>
       </c>
@@ -1937,7 +1937,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>83</v>
       </c>
@@ -1954,7 +1954,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>84</v>
       </c>
@@ -1971,7 +1971,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>86</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>88</v>
       </c>
@@ -2005,7 +2005,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>86</v>
       </c>
@@ -2022,7 +2022,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>88</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>90</v>
       </c>
@@ -2056,7 +2056,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>92</v>
       </c>
@@ -2073,7 +2073,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>93</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>90</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>94</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>96</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>97</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>99</v>
       </c>
@@ -2175,7 +2175,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>97</v>
       </c>
@@ -2192,7 +2192,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>101</v>
       </c>
@@ -2209,7 +2209,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>96</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>103</v>
       </c>
@@ -2243,7 +2243,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>105</v>
       </c>
@@ -2260,7 +2260,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>106</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>107</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>109</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>111</v>
       </c>
@@ -2328,7 +2328,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>113</v>
       </c>
@@ -2345,7 +2345,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>115</v>
       </c>
@@ -2362,7 +2362,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>107</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>109</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>113</v>
       </c>
@@ -2413,7 +2413,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>117</v>
       </c>
@@ -2430,7 +2430,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>119</v>
       </c>

</xml_diff>